<commit_message>
Verifica settimanale: 127 upgrade doppio controllo, log e stato aggiornati
Completa la verifica settimanale iniziata nel commit precedente (71
duplicati marcati). Doppio controllo indipendente (8 agenti paralleli,
WebSearch) su 177 righe DA VERIFICARE UMANAMENTE nei 70 file nuovi non
duplicati: 127 promosse a "VERIFICATA AI - doppio controllo
(21/09/2026)", 49 lasciate invariate per esito ambiguo, 1 lasciata
invariata per esito NON_CONFERMATA (nessun declassamento, nessuna
promozione senza conferma reale e indipendente).

Aggiornati weekly_verify_state.json (last_run_at, 70 nuovi file
processati) e weekly_verify_log.md con il resoconto del run, inclusi i
dettagli sulla guardia anti-falsi-positivi per catene multi-filiale
introdotta nella deduplica.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HLAeHJBUm8eZJoqNiASFPU
</commit_message>
<xml_diff>
--- a/output/2026-09-14_18_Croazia_Licko-senjska_Utensilerie_e_Macchine_Utensili.xlsx
+++ b/output/2026-09-14_18_Croazia_Licko-senjska_Utensilerie_e_Macchine_Utensili.xlsx
@@ -496,7 +496,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (21/09/2026)</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (21/09/2026)</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>DA VERIFICARE UMANAMENTE</t>
+          <t>VERIFICATA AI - doppio controllo (21/09/2026)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Verifica settimanale: deduplica globale cross-file (58 duplicati marcati)
Deduplica ricostruita con union-find su tutto il corpus (265 file, ~1960
righe nello schema di verifica). Match per nome esatto normalizzato e per
URL (dominio+path), con guardie anti-falso-positivo: stesso paese+regione
del nome file, conflitto nome-proprietario ("di <Nome Cognome>") e
conflitto di sede/filiale esplicita nel nome azienda (es. catene come
Pevex, Eurocolumbus, Sonepar, RemaTarlazzi, Strano, Garofoli con piu'
punti vendita sullo stesso dominio corporate non vengono accorpate).
Nessuna riga cancellata; solo annotazione "[DUPLICATO - vedi anche: ...]"
nel campo note delle occorrenze non canoniche. Annotazioni gia' presenti
da run precedenti lasciate invariate (nessun capovolgimento retroattivo).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V1d3BH14wLEVTJJVMB11Ey
</commit_message>
<xml_diff>
--- a/output/2026-09-14_18_Croazia_Licko-senjska_Utensilerie_e_Macchine_Utensili.xlsx
+++ b/output/2026-09-14_18_Croazia_Licko-senjska_Utensilerie_e_Macchine_Utensili.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Azienda verificata (sito ufficiale, tvrtke.hr, kompass.com). Attivo dal 1990, sede a Kaniža 5 e punto vendita ingrosso a Kralja Zvonimira 14, Gospić, oltre a Lički Osik. Attività principale: materiale edile, con reparto dedicato a 'građevinski alati' (utensili/attrezzi da costruzione) e ferramenta tecnica. Profilo B2B/B2C misto.</t>
+          <t>Azienda verificata (sito ufficiale, tvrtke.hr, kompass.com). Attivo dal 1990, sede a Kaniža 5 e punto vendita ingrosso a Kralja Zvonimira 14, Gospić, oltre a Lički Osik. Attività principale: materiale edile, con reparto dedicato a 'građevinski alati' (utensili/attrezzi da costruzione) e ferramenta tecnica. Profilo B2B/B2C misto. [DUPLICATO — vedi anche: 2026-09-14_03_Croazia_Licko-senjska_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -533,7 +533,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Azienda verificata (sito ufficiale, fininfo.hr, companywall.hr). Concessionario/rivenditore autorizzato Husqvarna e STIHL: vendita e assistenza di macchine e utensili motorizzati (motoseghe, decespugliatori, tosaerba, generatori, idropulitrici) per agricoltura, giardinaggio e forestazione. 3 punti vendita + magazzino ingrosso a Lički Osik.</t>
+          <t>Azienda verificata (sito ufficiale, fininfo.hr, companywall.hr). Concessionario/rivenditore autorizzato Husqvarna e STIHL: vendita e assistenza di macchine e utensili motorizzati (motoseghe, decespugliatori, tosaerba, generatori, idropulitrici) per agricoltura, giardinaggio e forestazione. 3 punti vendita + magazzino ingrosso a Lički Osik. [DUPLICATO — vedi anche: 2026-09-14_03_Croazia_Licko-senjska_Cleaning.xlsx]</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">

</xml_diff>